<commit_message>
Impl. OPL/OPLL drum kits
</commit_message>
<xml_diff>
--- a/banks/preset_bank_profile.xlsx
+++ b/banks/preset_bank_profile.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16920" windowHeight="8700" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16920" windowHeight="8700"/>
   </bookViews>
   <sheets>
     <sheet name="Patch Banks" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="174">
   <si>
     <t>CC#32</t>
     <phoneticPr fontId="1"/>
@@ -427,10 +427,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>OPLL ROM Patched</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>&lt;builtin&gt;</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -670,6 +666,22 @@
   </si>
   <si>
     <t># generate with similar to OPLL built-in</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OPLL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OPLL Built-In</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Built-In with performance</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t># generate skeleton, role=builtin_swpatch_meta</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1000,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
@@ -1055,7 +1067,7 @@
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1111,7 +1123,7 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1655,7 +1667,7 @@
         <v>48</v>
       </c>
       <c r="E39" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1805,10 +1817,10 @@
         <v>107</v>
       </c>
       <c r="D48" t="s">
+        <v>171</v>
+      </c>
+      <c r="E48" t="s">
         <v>108</v>
-      </c>
-      <c r="E48" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1819,13 +1831,13 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
+        <v>109</v>
+      </c>
+      <c r="D49" t="s">
         <v>110</v>
       </c>
-      <c r="D49" t="s">
-        <v>111</v>
-      </c>
       <c r="E49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1836,30 +1848,30 @@
         <v>2</v>
       </c>
       <c r="C50" t="s">
+        <v>113</v>
+      </c>
+      <c r="D50" t="s">
         <v>114</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>115</v>
-      </c>
-      <c r="E50" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C51" t="s">
-        <v>64</v>
+        <v>170</v>
       </c>
       <c r="D51" t="s">
-        <v>77</v>
+        <v>172</v>
       </c>
       <c r="E51" t="s">
-        <v>65</v>
+        <v>173</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1867,16 +1879,16 @@
         <v>48</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C52" t="s">
         <v>64</v>
       </c>
       <c r="D52" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="E52" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1884,16 +1896,16 @@
         <v>48</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="s">
         <v>64</v>
       </c>
       <c r="D53" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E53" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1901,16 +1913,16 @@
         <v>48</v>
       </c>
       <c r="B54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C54" t="s">
         <v>64</v>
       </c>
       <c r="D54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E54" t="s">
-        <v>118</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1918,16 +1930,16 @@
         <v>48</v>
       </c>
       <c r="B55">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" t="s">
         <v>64</v>
       </c>
       <c r="D55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E55" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -1935,16 +1947,16 @@
         <v>48</v>
       </c>
       <c r="B56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
         <v>64</v>
       </c>
       <c r="D56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1952,16 +1964,16 @@
         <v>48</v>
       </c>
       <c r="B57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C57" t="s">
         <v>64</v>
       </c>
       <c r="D57" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1969,16 +1981,16 @@
         <v>48</v>
       </c>
       <c r="B58">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C58" t="s">
         <v>64</v>
       </c>
       <c r="D58" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E58" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -1986,16 +1998,16 @@
         <v>48</v>
       </c>
       <c r="B59">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
         <v>64</v>
       </c>
       <c r="D59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -2003,33 +2015,33 @@
         <v>48</v>
       </c>
       <c r="B60">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="C60" t="s">
         <v>64</v>
       </c>
       <c r="D60" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E60" t="s">
-        <v>51</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
+        <v>48</v>
+      </c>
+      <c r="B61">
+        <v>112</v>
+      </c>
+      <c r="C61" t="s">
         <v>64</v>
       </c>
-      <c r="B61">
-        <v>0</v>
-      </c>
-      <c r="C61" t="s">
-        <v>120</v>
-      </c>
       <c r="D61" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="E61" t="s">
-        <v>122</v>
+        <v>51</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
@@ -2037,16 +2049,16 @@
         <v>64</v>
       </c>
       <c r="B62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C62" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D62" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E62" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2054,16 +2066,16 @@
         <v>64</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" t="s">
+        <v>122</v>
+      </c>
+      <c r="D63" t="s">
         <v>123</v>
       </c>
-      <c r="D63" t="s">
-        <v>128</v>
-      </c>
       <c r="E63" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -2071,47 +2083,47 @@
         <v>64</v>
       </c>
       <c r="B64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D64" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E64" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="B65">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C65" t="s">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="D65" t="s">
-        <v>168</v>
+        <v>128</v>
+      </c>
+      <c r="E65" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B66">
         <v>0</v>
       </c>
       <c r="C66" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D66" t="s">
-        <v>163</v>
-      </c>
-      <c r="E66" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -2119,16 +2131,33 @@
         <v>84</v>
       </c>
       <c r="B67">
+        <v>0</v>
+      </c>
+      <c r="C67" t="s">
+        <v>161</v>
+      </c>
+      <c r="D67" t="s">
+        <v>162</v>
+      </c>
+      <c r="E67" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>84</v>
+      </c>
+      <c r="B68">
         <v>1</v>
       </c>
-      <c r="C67" t="s">
-        <v>162</v>
-      </c>
-      <c r="D67" t="s">
-        <v>165</v>
-      </c>
-      <c r="E67" t="s">
+      <c r="C68" t="s">
+        <v>161</v>
+      </c>
+      <c r="D68" t="s">
         <v>164</v>
+      </c>
+      <c r="E68" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2149,13 +2178,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" t="s">
         <v>130</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>131</v>
-      </c>
-      <c r="C1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2163,10 +2192,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -2174,10 +2203,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2185,10 +2214,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" t="s">
         <v>134</v>
-      </c>
-      <c r="C4" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2196,10 +2225,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -2207,10 +2236,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" t="s">
         <v>139</v>
-      </c>
-      <c r="C6" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2218,10 +2247,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" t="s">
         <v>141</v>
-      </c>
-      <c r="C7" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2229,10 +2258,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" t="s">
         <v>143</v>
-      </c>
-      <c r="C8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -2240,10 +2269,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" t="s">
         <v>145</v>
-      </c>
-      <c r="C9" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2251,10 +2280,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" t="s">
         <v>147</v>
-      </c>
-      <c r="C10" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2262,10 +2291,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" t="s">
         <v>149</v>
-      </c>
-      <c r="C11" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2273,10 +2302,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" t="s">
         <v>151</v>
-      </c>
-      <c r="C12" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -2284,10 +2313,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" t="s">
         <v>169</v>
-      </c>
-      <c r="C13" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -2295,10 +2324,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C14" t="s">
         <v>153</v>
-      </c>
-      <c r="C14" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2306,10 +2335,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C15" t="s">
         <v>155</v>
-      </c>
-      <c r="C15" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -2317,10 +2346,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" t="s">
         <v>157</v>
-      </c>
-      <c r="C16" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -2328,10 +2357,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>